<commit_message>
Sicurezza e privacy, secondo e terzo giro (portachiavi solo su questo dispositivo, lettore e apertura dei file più sicuri, firma Android obbligatoria per le release, CSP del selettore di Drive, email personali tolte dal database, controllo della copia pubblica più completo, avvio della registrazione dal widget protetto); widget Android ridisegnati con avvio della registrazione dal widget; Windows: niente schermo nero al ripristino e chiusura immediata con la X
</commit_message>
<xml_diff>
--- a/app/test/fixtures/office/foglio.xlsx
+++ b/app/test/fixtures/office/foglio.xlsx
@@ -3,11 +3,6 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\simon\AppData\Local\Temp\claude\D--University-Notes\0e1973a7-21aa-4a45-b9ef-77200eb6c84a\scratchpad\agente2\office\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="8_{E391DBA7-316B-452F-8AC5-344F3053ACF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{71351A28-A73D-485A-A0D4-9E2B388CF68D}"/>

</xml_diff>